<commit_message>
:bat: modif manually taxo table before split + keep Mothers_0days for compo
</commit_message>
<xml_diff>
--- a/data/derived_data/2_RarefyData/Dataset_1/ps_ITS_filt_Dataset_1_tax_table.xlsx
+++ b/data/derived_data/2_RarefyData/Dataset_1/ps_ITS_filt_Dataset_1_tax_table.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="215" uniqueCount="215">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="229" uniqueCount="229">
   <si>
     <t xml:space="preserve"/>
   </si>
@@ -95,6 +95,24 @@
     <t xml:space="preserve">Dothiora prunorum</t>
   </si>
   <si>
+    <t xml:space="preserve">Cluster_103</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Saccharomycetes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Saccharomycetales</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Phaffomycetaceae</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Wickerhamomyces</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Wickerhamomyces pijperi</t>
+  </si>
+  <si>
     <t xml:space="preserve">Cluster_105</t>
   </si>
   <si>
@@ -122,6 +140,12 @@
     <t xml:space="preserve">Cluster_117</t>
   </si>
   <si>
+    <t xml:space="preserve">Cluster_12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pichia nakasei</t>
+  </si>
+  <si>
     <t xml:space="preserve">Cluster_123</t>
   </si>
   <si>
@@ -239,12 +263,6 @@
     <t xml:space="preserve">Cluster_18</t>
   </si>
   <si>
-    <t xml:space="preserve">Saccharomycetes</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Saccharomycetales</t>
-  </si>
-  <si>
     <t xml:space="preserve">Saccharomycodaceae</t>
   </si>
   <si>
@@ -254,6 +272,24 @@
     <t xml:space="preserve">Cluster_182</t>
   </si>
   <si>
+    <t xml:space="preserve">Cluster_187</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Eurotiomycetes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Eurotiales</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aspergillaceae</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Penicillium</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Penicillium bialowiezense</t>
+  </si>
+  <si>
     <t xml:space="preserve">Cluster_188</t>
   </si>
   <si>
@@ -356,15 +392,6 @@
     <t xml:space="preserve">Cluster_29</t>
   </si>
   <si>
-    <t xml:space="preserve">Phaffomycetaceae</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Wickerhamomyces</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Wickerhamomyces pijperi</t>
-  </si>
-  <si>
     <t xml:space="preserve">Cluster_295</t>
   </si>
   <si>
@@ -380,18 +407,6 @@
     <t xml:space="preserve">Cluster_30</t>
   </si>
   <si>
-    <t xml:space="preserve">Eurotiomycetes</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Eurotiales</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Aspergillaceae</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Penicillium</t>
-  </si>
-  <si>
     <t xml:space="preserve">Penicillium brevicompactum</t>
   </si>
   <si>
@@ -428,6 +443,9 @@
     <t xml:space="preserve">Cluster_33</t>
   </si>
   <si>
+    <t xml:space="preserve">Cluster_34</t>
+  </si>
+  <si>
     <t xml:space="preserve">Cluster_340</t>
   </si>
   <si>
@@ -497,6 +515,27 @@
     <t xml:space="preserve">Podosphaera</t>
   </si>
   <si>
+    <t xml:space="preserve">Cluster_422</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mucoromycota</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mucoromycetes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mucorales</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mucoraceae</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mucor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mucor circinelloides</t>
+  </si>
+  <si>
     <t xml:space="preserve">Cluster_423</t>
   </si>
   <si>
@@ -618,6 +657,9 @@
   </si>
   <si>
     <t xml:space="preserve">Cluster_82</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cluster_83</t>
   </si>
   <si>
     <t xml:space="preserve">Cluster_85</t>
@@ -1094,56 +1136,56 @@
         <v>27</v>
       </c>
       <c r="B5" t="s">
-        <v>28</v>
+        <v>9</v>
       </c>
       <c r="C5" t="s">
-        <v>28</v>
+        <v>10</v>
       </c>
       <c r="D5" t="s">
         <v>28</v>
       </c>
       <c r="E5" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F5" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="G5" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="H5" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="B6" t="s">
-        <v>9</v>
+        <v>34</v>
       </c>
       <c r="C6" t="s">
-        <v>10</v>
+        <v>34</v>
       </c>
       <c r="D6" t="s">
-        <v>11</v>
+        <v>34</v>
       </c>
       <c r="E6" t="s">
-        <v>17</v>
+        <v>34</v>
       </c>
       <c r="F6" t="s">
-        <v>18</v>
+        <v>34</v>
       </c>
       <c r="G6" t="s">
-        <v>19</v>
+        <v>34</v>
       </c>
       <c r="H6" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="B7" t="s">
         <v>9</v>
@@ -1164,56 +1206,56 @@
         <v>19</v>
       </c>
       <c r="H7" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="B8" t="s">
-        <v>28</v>
+        <v>9</v>
       </c>
       <c r="C8" t="s">
-        <v>28</v>
+        <v>10</v>
       </c>
       <c r="D8" t="s">
-        <v>28</v>
+        <v>11</v>
       </c>
       <c r="E8" t="s">
-        <v>28</v>
+        <v>17</v>
       </c>
       <c r="F8" t="s">
-        <v>28</v>
+        <v>18</v>
       </c>
       <c r="G8" t="s">
-        <v>28</v>
+        <v>19</v>
       </c>
       <c r="H8" t="s">
-        <v>28</v>
+        <v>37</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="B9" t="s">
-        <v>9</v>
+        <v>34</v>
       </c>
       <c r="C9" t="s">
-        <v>10</v>
+        <v>34</v>
       </c>
       <c r="D9" t="s">
-        <v>11</v>
+        <v>34</v>
       </c>
       <c r="E9" t="s">
-        <v>17</v>
+        <v>34</v>
       </c>
       <c r="F9" t="s">
-        <v>18</v>
+        <v>34</v>
       </c>
       <c r="G9" t="s">
-        <v>19</v>
+        <v>34</v>
       </c>
       <c r="H9" t="s">
         <v>34</v>
@@ -1221,7 +1263,7 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="B10" t="s">
         <v>9</v>
@@ -1242,33 +1284,33 @@
         <v>19</v>
       </c>
       <c r="H10" t="s">
-        <v>31</v>
+        <v>40</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="B11" t="s">
         <v>9</v>
       </c>
       <c r="C11" t="s">
+        <v>10</v>
+      </c>
+      <c r="D11" t="s">
+        <v>11</v>
+      </c>
+      <c r="E11" t="s">
+        <v>17</v>
+      </c>
+      <c r="F11" t="s">
+        <v>18</v>
+      </c>
+      <c r="G11" t="s">
+        <v>19</v>
+      </c>
+      <c r="H11" t="s">
         <v>37</v>
-      </c>
-      <c r="D11" t="s">
-        <v>38</v>
-      </c>
-      <c r="E11" t="s">
-        <v>39</v>
-      </c>
-      <c r="F11" t="s">
-        <v>40</v>
-      </c>
-      <c r="G11" t="s">
-        <v>41</v>
-      </c>
-      <c r="H11" t="s">
-        <v>28</v>
       </c>
     </row>
     <row r="12">
@@ -1285,47 +1327,47 @@
         <v>11</v>
       </c>
       <c r="E12" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="F12" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="G12" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="H12" t="s">
-        <v>28</v>
+        <v>43</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B13" t="s">
         <v>9</v>
       </c>
       <c r="C13" t="s">
-        <v>10</v>
+        <v>45</v>
       </c>
       <c r="D13" t="s">
-        <v>11</v>
+        <v>46</v>
       </c>
       <c r="E13" t="s">
-        <v>17</v>
+        <v>47</v>
       </c>
       <c r="F13" t="s">
-        <v>18</v>
+        <v>48</v>
       </c>
       <c r="G13" t="s">
-        <v>19</v>
+        <v>49</v>
       </c>
       <c r="H13" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>44</v>
+        <v>50</v>
       </c>
       <c r="B14" t="s">
         <v>9</v>
@@ -1334,24 +1376,24 @@
         <v>10</v>
       </c>
       <c r="D14" t="s">
-        <v>45</v>
+        <v>11</v>
       </c>
       <c r="E14" t="s">
-        <v>46</v>
+        <v>17</v>
       </c>
       <c r="F14" t="s">
-        <v>47</v>
+        <v>18</v>
       </c>
       <c r="G14" t="s">
-        <v>48</v>
+        <v>19</v>
       </c>
       <c r="H14" t="s">
-        <v>49</v>
+        <v>34</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B15" t="s">
         <v>9</v>
@@ -1360,50 +1402,50 @@
         <v>10</v>
       </c>
       <c r="D15" t="s">
-        <v>22</v>
+        <v>11</v>
       </c>
       <c r="E15" t="s">
-        <v>51</v>
+        <v>17</v>
       </c>
       <c r="F15" t="s">
-        <v>52</v>
+        <v>18</v>
       </c>
       <c r="G15" t="s">
-        <v>53</v>
+        <v>19</v>
       </c>
       <c r="H15" t="s">
-        <v>28</v>
+        <v>37</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
+        <v>52</v>
+      </c>
+      <c r="B16" t="s">
+        <v>9</v>
+      </c>
+      <c r="C16" t="s">
+        <v>10</v>
+      </c>
+      <c r="D16" t="s">
+        <v>53</v>
+      </c>
+      <c r="E16" t="s">
         <v>54</v>
       </c>
-      <c r="B16" t="s">
-        <v>9</v>
-      </c>
-      <c r="C16" t="s">
-        <v>10</v>
-      </c>
-      <c r="D16" t="s">
-        <v>11</v>
-      </c>
-      <c r="E16" t="s">
-        <v>17</v>
-      </c>
       <c r="F16" t="s">
-        <v>18</v>
+        <v>55</v>
       </c>
       <c r="G16" t="s">
-        <v>19</v>
+        <v>56</v>
       </c>
       <c r="H16" t="s">
-        <v>34</v>
+        <v>57</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="B17" t="s">
         <v>9</v>
@@ -1412,50 +1454,50 @@
         <v>10</v>
       </c>
       <c r="D17" t="s">
-        <v>11</v>
+        <v>22</v>
       </c>
       <c r="E17" t="s">
-        <v>17</v>
+        <v>59</v>
       </c>
       <c r="F17" t="s">
-        <v>18</v>
+        <v>60</v>
       </c>
       <c r="G17" t="s">
-        <v>19</v>
+        <v>61</v>
       </c>
       <c r="H17" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>56</v>
+        <v>62</v>
       </c>
       <c r="B18" t="s">
         <v>9</v>
       </c>
       <c r="C18" t="s">
-        <v>37</v>
+        <v>10</v>
       </c>
       <c r="D18" t="s">
-        <v>38</v>
+        <v>11</v>
       </c>
       <c r="E18" t="s">
-        <v>39</v>
+        <v>17</v>
       </c>
       <c r="F18" t="s">
-        <v>28</v>
+        <v>18</v>
       </c>
       <c r="G18" t="s">
-        <v>28</v>
+        <v>19</v>
       </c>
       <c r="H18" t="s">
-        <v>28</v>
+        <v>40</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>57</v>
+        <v>63</v>
       </c>
       <c r="B19" t="s">
         <v>9</v>
@@ -1464,76 +1506,76 @@
         <v>10</v>
       </c>
       <c r="D19" t="s">
-        <v>22</v>
+        <v>11</v>
       </c>
       <c r="E19" t="s">
-        <v>58</v>
+        <v>17</v>
       </c>
       <c r="F19" t="s">
-        <v>59</v>
+        <v>18</v>
       </c>
       <c r="G19" t="s">
-        <v>60</v>
+        <v>19</v>
       </c>
       <c r="H19" t="s">
-        <v>61</v>
+        <v>37</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="B20" t="s">
         <v>9</v>
       </c>
       <c r="C20" t="s">
-        <v>10</v>
+        <v>45</v>
       </c>
       <c r="D20" t="s">
-        <v>22</v>
+        <v>46</v>
       </c>
       <c r="E20" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="F20" t="s">
-        <v>52</v>
+        <v>34</v>
       </c>
       <c r="G20" t="s">
-        <v>53</v>
+        <v>34</v>
       </c>
       <c r="H20" t="s">
-        <v>63</v>
+        <v>34</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B21" t="s">
         <v>9</v>
       </c>
       <c r="C21" t="s">
-        <v>28</v>
+        <v>10</v>
       </c>
       <c r="D21" t="s">
-        <v>28</v>
+        <v>22</v>
       </c>
       <c r="E21" t="s">
-        <v>28</v>
+        <v>66</v>
       </c>
       <c r="F21" t="s">
-        <v>28</v>
+        <v>67</v>
       </c>
       <c r="G21" t="s">
-        <v>28</v>
+        <v>68</v>
       </c>
       <c r="H21" t="s">
-        <v>28</v>
+        <v>69</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="B22" t="s">
         <v>9</v>
@@ -1545,47 +1587,47 @@
         <v>22</v>
       </c>
       <c r="E22" t="s">
-        <v>51</v>
+        <v>59</v>
       </c>
       <c r="F22" t="s">
-        <v>52</v>
+        <v>60</v>
       </c>
       <c r="G22" t="s">
-        <v>28</v>
+        <v>61</v>
       </c>
       <c r="H22" t="s">
-        <v>28</v>
+        <v>71</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="B23" t="s">
         <v>9</v>
       </c>
       <c r="C23" t="s">
-        <v>10</v>
+        <v>34</v>
       </c>
       <c r="D23" t="s">
-        <v>11</v>
+        <v>34</v>
       </c>
       <c r="E23" t="s">
-        <v>17</v>
+        <v>34</v>
       </c>
       <c r="F23" t="s">
-        <v>18</v>
+        <v>34</v>
       </c>
       <c r="G23" t="s">
-        <v>19</v>
+        <v>34</v>
       </c>
       <c r="H23" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="s">
-        <v>67</v>
+        <v>73</v>
       </c>
       <c r="B24" t="s">
         <v>9</v>
@@ -1597,125 +1639,125 @@
         <v>22</v>
       </c>
       <c r="E24" t="s">
-        <v>51</v>
+        <v>59</v>
       </c>
       <c r="F24" t="s">
-        <v>52</v>
+        <v>60</v>
       </c>
       <c r="G24" t="s">
-        <v>68</v>
+        <v>34</v>
       </c>
       <c r="H24" t="s">
-        <v>69</v>
+        <v>34</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="B25" t="s">
         <v>9</v>
       </c>
       <c r="C25" t="s">
-        <v>37</v>
+        <v>10</v>
       </c>
       <c r="D25" t="s">
-        <v>38</v>
+        <v>11</v>
       </c>
       <c r="E25" t="s">
-        <v>39</v>
+        <v>17</v>
       </c>
       <c r="F25" t="s">
-        <v>71</v>
+        <v>18</v>
       </c>
       <c r="G25" t="s">
-        <v>72</v>
+        <v>19</v>
       </c>
       <c r="H25" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="B26" t="s">
         <v>9</v>
       </c>
       <c r="C26" t="s">
-        <v>37</v>
+        <v>10</v>
       </c>
       <c r="D26" t="s">
-        <v>38</v>
+        <v>22</v>
       </c>
       <c r="E26" t="s">
-        <v>39</v>
+        <v>59</v>
       </c>
       <c r="F26" t="s">
-        <v>28</v>
+        <v>60</v>
       </c>
       <c r="G26" t="s">
-        <v>28</v>
+        <v>76</v>
       </c>
       <c r="H26" t="s">
-        <v>28</v>
+        <v>77</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="B27" t="s">
         <v>9</v>
       </c>
       <c r="C27" t="s">
-        <v>10</v>
+        <v>45</v>
       </c>
       <c r="D27" t="s">
-        <v>75</v>
+        <v>46</v>
       </c>
       <c r="E27" t="s">
-        <v>76</v>
+        <v>47</v>
       </c>
       <c r="F27" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="G27" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="H27" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="B28" t="s">
         <v>9</v>
       </c>
       <c r="C28" t="s">
-        <v>28</v>
+        <v>45</v>
       </c>
       <c r="D28" t="s">
-        <v>28</v>
+        <v>46</v>
       </c>
       <c r="E28" t="s">
-        <v>28</v>
+        <v>47</v>
       </c>
       <c r="F28" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="G28" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="H28" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B29" t="s">
         <v>9</v>
@@ -1724,50 +1766,50 @@
         <v>10</v>
       </c>
       <c r="D29" t="s">
-        <v>45</v>
+        <v>28</v>
       </c>
       <c r="E29" t="s">
-        <v>46</v>
+        <v>29</v>
       </c>
       <c r="F29" t="s">
-        <v>47</v>
+        <v>83</v>
       </c>
       <c r="G29" t="s">
-        <v>48</v>
+        <v>84</v>
       </c>
       <c r="H29" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="B30" t="s">
         <v>9</v>
       </c>
       <c r="C30" t="s">
-        <v>10</v>
+        <v>34</v>
       </c>
       <c r="D30" t="s">
-        <v>11</v>
+        <v>34</v>
       </c>
       <c r="E30" t="s">
-        <v>12</v>
+        <v>34</v>
       </c>
       <c r="F30" t="s">
-        <v>13</v>
+        <v>34</v>
       </c>
       <c r="G30" t="s">
-        <v>14</v>
+        <v>34</v>
       </c>
       <c r="H30" t="s">
-        <v>15</v>
+        <v>34</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="B31" t="s">
         <v>9</v>
@@ -1776,24 +1818,24 @@
         <v>10</v>
       </c>
       <c r="D31" t="s">
-        <v>11</v>
+        <v>87</v>
       </c>
       <c r="E31" t="s">
-        <v>17</v>
+        <v>88</v>
       </c>
       <c r="F31" t="s">
-        <v>18</v>
+        <v>89</v>
       </c>
       <c r="G31" t="s">
-        <v>19</v>
+        <v>90</v>
       </c>
       <c r="H31" t="s">
-        <v>31</v>
+        <v>91</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="s">
-        <v>83</v>
+        <v>92</v>
       </c>
       <c r="B32" t="s">
         <v>9</v>
@@ -1802,76 +1844,76 @@
         <v>10</v>
       </c>
       <c r="D32" t="s">
-        <v>84</v>
+        <v>53</v>
       </c>
       <c r="E32" t="s">
-        <v>85</v>
+        <v>54</v>
       </c>
       <c r="F32" t="s">
-        <v>86</v>
+        <v>55</v>
       </c>
       <c r="G32" t="s">
-        <v>87</v>
+        <v>56</v>
       </c>
       <c r="H32" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="s">
-        <v>88</v>
+        <v>93</v>
       </c>
       <c r="B33" t="s">
         <v>9</v>
       </c>
       <c r="C33" t="s">
-        <v>37</v>
+        <v>10</v>
       </c>
       <c r="D33" t="s">
-        <v>38</v>
+        <v>11</v>
       </c>
       <c r="E33" t="s">
-        <v>39</v>
+        <v>12</v>
       </c>
       <c r="F33" t="s">
-        <v>40</v>
+        <v>13</v>
       </c>
       <c r="G33" t="s">
-        <v>41</v>
+        <v>14</v>
       </c>
       <c r="H33" t="s">
-        <v>89</v>
+        <v>15</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="B34" t="s">
         <v>9</v>
       </c>
       <c r="C34" t="s">
+        <v>10</v>
+      </c>
+      <c r="D34" t="s">
+        <v>11</v>
+      </c>
+      <c r="E34" t="s">
+        <v>17</v>
+      </c>
+      <c r="F34" t="s">
+        <v>18</v>
+      </c>
+      <c r="G34" t="s">
+        <v>19</v>
+      </c>
+      <c r="H34" t="s">
         <v>37</v>
-      </c>
-      <c r="D34" t="s">
-        <v>91</v>
-      </c>
-      <c r="E34" t="s">
-        <v>92</v>
-      </c>
-      <c r="F34" t="s">
-        <v>28</v>
-      </c>
-      <c r="G34" t="s">
-        <v>28</v>
-      </c>
-      <c r="H34" t="s">
-        <v>28</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="B35" t="s">
         <v>9</v>
@@ -1880,76 +1922,76 @@
         <v>10</v>
       </c>
       <c r="D35" t="s">
-        <v>22</v>
+        <v>96</v>
       </c>
       <c r="E35" t="s">
-        <v>58</v>
+        <v>97</v>
       </c>
       <c r="F35" t="s">
-        <v>59</v>
+        <v>98</v>
       </c>
       <c r="G35" t="s">
-        <v>94</v>
+        <v>99</v>
       </c>
       <c r="H35" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="B36" t="s">
-        <v>28</v>
+        <v>9</v>
       </c>
       <c r="C36" t="s">
-        <v>28</v>
+        <v>45</v>
       </c>
       <c r="D36" t="s">
-        <v>28</v>
+        <v>46</v>
       </c>
       <c r="E36" t="s">
-        <v>28</v>
+        <v>47</v>
       </c>
       <c r="F36" t="s">
-        <v>28</v>
+        <v>48</v>
       </c>
       <c r="G36" t="s">
-        <v>28</v>
+        <v>49</v>
       </c>
       <c r="H36" t="s">
-        <v>28</v>
+        <v>101</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="s">
-        <v>96</v>
+        <v>102</v>
       </c>
       <c r="B37" t="s">
         <v>9</v>
       </c>
       <c r="C37" t="s">
-        <v>10</v>
+        <v>45</v>
       </c>
       <c r="D37" t="s">
-        <v>11</v>
+        <v>103</v>
       </c>
       <c r="E37" t="s">
-        <v>17</v>
+        <v>104</v>
       </c>
       <c r="F37" t="s">
-        <v>18</v>
+        <v>34</v>
       </c>
       <c r="G37" t="s">
-        <v>19</v>
+        <v>34</v>
       </c>
       <c r="H37" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="s">
-        <v>97</v>
+        <v>105</v>
       </c>
       <c r="B38" t="s">
         <v>9</v>
@@ -1961,99 +2003,99 @@
         <v>22</v>
       </c>
       <c r="E38" t="s">
-        <v>51</v>
+        <v>66</v>
       </c>
       <c r="F38" t="s">
-        <v>52</v>
+        <v>67</v>
       </c>
       <c r="G38" t="s">
-        <v>53</v>
+        <v>106</v>
       </c>
       <c r="H38" t="s">
-        <v>98</v>
+        <v>34</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="s">
-        <v>99</v>
+        <v>107</v>
       </c>
       <c r="B39" t="s">
-        <v>9</v>
+        <v>34</v>
       </c>
       <c r="C39" t="s">
-        <v>10</v>
+        <v>34</v>
       </c>
       <c r="D39" t="s">
-        <v>11</v>
+        <v>34</v>
       </c>
       <c r="E39" t="s">
-        <v>17</v>
+        <v>34</v>
       </c>
       <c r="F39" t="s">
-        <v>18</v>
+        <v>34</v>
       </c>
       <c r="G39" t="s">
-        <v>19</v>
+        <v>34</v>
       </c>
       <c r="H39" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="s">
-        <v>100</v>
+        <v>108</v>
       </c>
       <c r="B40" t="s">
         <v>9</v>
       </c>
       <c r="C40" t="s">
-        <v>28</v>
+        <v>10</v>
       </c>
       <c r="D40" t="s">
-        <v>28</v>
+        <v>11</v>
       </c>
       <c r="E40" t="s">
-        <v>28</v>
+        <v>17</v>
       </c>
       <c r="F40" t="s">
-        <v>28</v>
+        <v>18</v>
       </c>
       <c r="G40" t="s">
-        <v>28</v>
+        <v>19</v>
       </c>
       <c r="H40" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="s">
-        <v>101</v>
+        <v>109</v>
       </c>
       <c r="B41" t="s">
         <v>9</v>
       </c>
       <c r="C41" t="s">
-        <v>37</v>
+        <v>10</v>
       </c>
       <c r="D41" t="s">
-        <v>38</v>
+        <v>22</v>
       </c>
       <c r="E41" t="s">
-        <v>39</v>
+        <v>59</v>
       </c>
       <c r="F41" t="s">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="G41" t="s">
-        <v>102</v>
+        <v>61</v>
       </c>
       <c r="H41" t="s">
-        <v>28</v>
+        <v>110</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="s">
-        <v>103</v>
+        <v>111</v>
       </c>
       <c r="B42" t="s">
         <v>9</v>
@@ -2062,76 +2104,76 @@
         <v>10</v>
       </c>
       <c r="D42" t="s">
-        <v>22</v>
+        <v>11</v>
       </c>
       <c r="E42" t="s">
-        <v>58</v>
+        <v>17</v>
       </c>
       <c r="F42" t="s">
-        <v>59</v>
+        <v>18</v>
       </c>
       <c r="G42" t="s">
-        <v>94</v>
+        <v>19</v>
       </c>
       <c r="H42" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="s">
-        <v>104</v>
+        <v>112</v>
       </c>
       <c r="B43" t="s">
         <v>9</v>
       </c>
       <c r="C43" t="s">
-        <v>10</v>
+        <v>34</v>
       </c>
       <c r="D43" t="s">
-        <v>22</v>
+        <v>34</v>
       </c>
       <c r="E43" t="s">
-        <v>51</v>
+        <v>34</v>
       </c>
       <c r="F43" t="s">
-        <v>52</v>
+        <v>34</v>
       </c>
       <c r="G43" t="s">
-        <v>53</v>
+        <v>34</v>
       </c>
       <c r="H43" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="s">
-        <v>105</v>
+        <v>113</v>
       </c>
       <c r="B44" t="s">
         <v>9</v>
       </c>
       <c r="C44" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="D44" t="s">
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="E44" t="s">
-        <v>106</v>
+        <v>47</v>
       </c>
       <c r="F44" t="s">
-        <v>107</v>
+        <v>48</v>
       </c>
       <c r="G44" t="s">
-        <v>108</v>
+        <v>114</v>
       </c>
       <c r="H44" t="s">
-        <v>109</v>
+        <v>34</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="s">
-        <v>110</v>
+        <v>115</v>
       </c>
       <c r="B45" t="s">
         <v>9</v>
@@ -2140,24 +2182,24 @@
         <v>10</v>
       </c>
       <c r="D45" t="s">
-        <v>11</v>
+        <v>22</v>
       </c>
       <c r="E45" t="s">
-        <v>17</v>
+        <v>66</v>
       </c>
       <c r="F45" t="s">
-        <v>18</v>
+        <v>67</v>
       </c>
       <c r="G45" t="s">
-        <v>19</v>
+        <v>106</v>
       </c>
       <c r="H45" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="s">
-        <v>111</v>
+        <v>116</v>
       </c>
       <c r="B46" t="s">
         <v>9</v>
@@ -2166,50 +2208,50 @@
         <v>10</v>
       </c>
       <c r="D46" t="s">
-        <v>11</v>
+        <v>22</v>
       </c>
       <c r="E46" t="s">
-        <v>17</v>
+        <v>59</v>
       </c>
       <c r="F46" t="s">
-        <v>18</v>
+        <v>60</v>
       </c>
       <c r="G46" t="s">
-        <v>19</v>
+        <v>61</v>
       </c>
       <c r="H46" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
       <c r="B47" t="s">
         <v>9</v>
       </c>
       <c r="C47" t="s">
-        <v>10</v>
+        <v>45</v>
       </c>
       <c r="D47" t="s">
-        <v>11</v>
+        <v>46</v>
       </c>
       <c r="E47" t="s">
-        <v>17</v>
+        <v>118</v>
       </c>
       <c r="F47" t="s">
-        <v>18</v>
+        <v>119</v>
       </c>
       <c r="G47" t="s">
-        <v>19</v>
+        <v>120</v>
       </c>
       <c r="H47" t="s">
-        <v>31</v>
+        <v>121</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="s">
-        <v>113</v>
+        <v>122</v>
       </c>
       <c r="B48" t="s">
         <v>9</v>
@@ -2218,24 +2260,24 @@
         <v>10</v>
       </c>
       <c r="D48" t="s">
-        <v>75</v>
+        <v>11</v>
       </c>
       <c r="E48" t="s">
-        <v>76</v>
+        <v>17</v>
       </c>
       <c r="F48" t="s">
-        <v>114</v>
+        <v>18</v>
       </c>
       <c r="G48" t="s">
-        <v>115</v>
+        <v>19</v>
       </c>
       <c r="H48" t="s">
-        <v>116</v>
+        <v>34</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="s">
-        <v>117</v>
+        <v>123</v>
       </c>
       <c r="B49" t="s">
         <v>9</v>
@@ -2244,24 +2286,24 @@
         <v>10</v>
       </c>
       <c r="D49" t="s">
-        <v>22</v>
+        <v>11</v>
       </c>
       <c r="E49" t="s">
-        <v>51</v>
+        <v>17</v>
       </c>
       <c r="F49" t="s">
-        <v>52</v>
+        <v>18</v>
       </c>
       <c r="G49" t="s">
-        <v>53</v>
+        <v>19</v>
       </c>
       <c r="H49" t="s">
-        <v>118</v>
+        <v>34</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="s">
-        <v>119</v>
+        <v>124</v>
       </c>
       <c r="B50" t="s">
         <v>9</v>
@@ -2273,21 +2315,21 @@
         <v>11</v>
       </c>
       <c r="E50" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="F50" t="s">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="G50" t="s">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="H50" t="s">
-        <v>120</v>
+        <v>37</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="B51" t="s">
         <v>9</v>
@@ -2296,50 +2338,50 @@
         <v>10</v>
       </c>
       <c r="D51" t="s">
-        <v>122</v>
+        <v>28</v>
       </c>
       <c r="E51" t="s">
-        <v>123</v>
+        <v>29</v>
       </c>
       <c r="F51" t="s">
-        <v>124</v>
+        <v>30</v>
       </c>
       <c r="G51" t="s">
-        <v>125</v>
+        <v>31</v>
       </c>
       <c r="H51" t="s">
-        <v>126</v>
+        <v>32</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="s">
+        <v>126</v>
+      </c>
+      <c r="B52" t="s">
+        <v>9</v>
+      </c>
+      <c r="C52" t="s">
+        <v>10</v>
+      </c>
+      <c r="D52" t="s">
+        <v>22</v>
+      </c>
+      <c r="E52" t="s">
+        <v>59</v>
+      </c>
+      <c r="F52" t="s">
+        <v>60</v>
+      </c>
+      <c r="G52" t="s">
+        <v>61</v>
+      </c>
+      <c r="H52" t="s">
         <v>127</v>
-      </c>
-      <c r="B52" t="s">
-        <v>9</v>
-      </c>
-      <c r="C52" t="s">
-        <v>37</v>
-      </c>
-      <c r="D52" t="s">
-        <v>128</v>
-      </c>
-      <c r="E52" t="s">
-        <v>129</v>
-      </c>
-      <c r="F52" t="s">
-        <v>130</v>
-      </c>
-      <c r="G52" t="s">
-        <v>131</v>
-      </c>
-      <c r="H52" t="s">
-        <v>132</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="s">
-        <v>133</v>
+        <v>128</v>
       </c>
       <c r="B53" t="s">
         <v>9</v>
@@ -2351,73 +2393,73 @@
         <v>11</v>
       </c>
       <c r="E53" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="F53" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="G53" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="H53" t="s">
-        <v>134</v>
+        <v>129</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="s">
-        <v>135</v>
+        <v>130</v>
       </c>
       <c r="B54" t="s">
-        <v>28</v>
+        <v>9</v>
       </c>
       <c r="C54" t="s">
-        <v>28</v>
+        <v>10</v>
       </c>
       <c r="D54" t="s">
-        <v>28</v>
+        <v>87</v>
       </c>
       <c r="E54" t="s">
-        <v>28</v>
+        <v>88</v>
       </c>
       <c r="F54" t="s">
-        <v>28</v>
+        <v>89</v>
       </c>
       <c r="G54" t="s">
-        <v>28</v>
+        <v>90</v>
       </c>
       <c r="H54" t="s">
-        <v>28</v>
+        <v>131</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="s">
+        <v>132</v>
+      </c>
+      <c r="B55" t="s">
+        <v>9</v>
+      </c>
+      <c r="C55" t="s">
+        <v>45</v>
+      </c>
+      <c r="D55" t="s">
+        <v>133</v>
+      </c>
+      <c r="E55" t="s">
+        <v>134</v>
+      </c>
+      <c r="F55" t="s">
+        <v>135</v>
+      </c>
+      <c r="G55" t="s">
         <v>136</v>
       </c>
-      <c r="B55" t="s">
-        <v>9</v>
-      </c>
-      <c r="C55" t="s">
-        <v>10</v>
-      </c>
-      <c r="D55" t="s">
-        <v>11</v>
-      </c>
-      <c r="E55" t="s">
-        <v>17</v>
-      </c>
-      <c r="F55" t="s">
-        <v>18</v>
-      </c>
-      <c r="G55" t="s">
-        <v>19</v>
-      </c>
       <c r="H55" t="s">
-        <v>31</v>
+        <v>137</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="B56" t="s">
         <v>9</v>
@@ -2438,38 +2480,38 @@
         <v>19</v>
       </c>
       <c r="H56" t="s">
-        <v>31</v>
+        <v>139</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="B57" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="C57" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="D57" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="E57" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="F57" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="G57" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="H57" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B58" t="s">
         <v>9</v>
@@ -2478,24 +2520,24 @@
         <v>10</v>
       </c>
       <c r="D58" t="s">
-        <v>22</v>
+        <v>11</v>
       </c>
       <c r="E58" t="s">
-        <v>140</v>
+        <v>17</v>
       </c>
       <c r="F58" t="s">
-        <v>141</v>
+        <v>18</v>
       </c>
       <c r="G58" t="s">
-        <v>142</v>
+        <v>19</v>
       </c>
       <c r="H58" t="s">
-        <v>143</v>
+        <v>37</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="B59" t="s">
         <v>9</v>
@@ -2516,90 +2558,90 @@
         <v>19</v>
       </c>
       <c r="H59" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="B60" t="s">
         <v>9</v>
       </c>
       <c r="C60" t="s">
-        <v>37</v>
+        <v>10</v>
       </c>
       <c r="D60" t="s">
-        <v>146</v>
+        <v>28</v>
       </c>
       <c r="E60" t="s">
-        <v>147</v>
+        <v>29</v>
       </c>
       <c r="F60" t="s">
-        <v>148</v>
+        <v>34</v>
       </c>
       <c r="G60" t="s">
-        <v>149</v>
+        <v>34</v>
       </c>
       <c r="H60" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="s">
-        <v>150</v>
+        <v>144</v>
       </c>
       <c r="B61" t="s">
-        <v>9</v>
+        <v>34</v>
       </c>
       <c r="C61" t="s">
-        <v>10</v>
+        <v>34</v>
       </c>
       <c r="D61" t="s">
-        <v>11</v>
+        <v>34</v>
       </c>
       <c r="E61" t="s">
-        <v>17</v>
+        <v>34</v>
       </c>
       <c r="F61" t="s">
-        <v>18</v>
+        <v>34</v>
       </c>
       <c r="G61" t="s">
-        <v>19</v>
+        <v>34</v>
       </c>
       <c r="H61" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="s">
-        <v>151</v>
+        <v>145</v>
       </c>
       <c r="B62" t="s">
-        <v>28</v>
+        <v>9</v>
       </c>
       <c r="C62" t="s">
-        <v>28</v>
+        <v>10</v>
       </c>
       <c r="D62" t="s">
-        <v>28</v>
+        <v>22</v>
       </c>
       <c r="E62" t="s">
-        <v>28</v>
+        <v>146</v>
       </c>
       <c r="F62" t="s">
-        <v>28</v>
+        <v>147</v>
       </c>
       <c r="G62" t="s">
-        <v>28</v>
+        <v>148</v>
       </c>
       <c r="H62" t="s">
-        <v>28</v>
+        <v>149</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="B63" t="s">
         <v>9</v>
@@ -2620,30 +2662,30 @@
         <v>19</v>
       </c>
       <c r="H63" t="s">
-        <v>20</v>
+        <v>37</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="s">
+        <v>151</v>
+      </c>
+      <c r="B64" t="s">
+        <v>9</v>
+      </c>
+      <c r="C64" t="s">
+        <v>45</v>
+      </c>
+      <c r="D64" t="s">
+        <v>152</v>
+      </c>
+      <c r="E64" t="s">
         <v>153</v>
       </c>
-      <c r="B64" t="s">
-        <v>9</v>
-      </c>
-      <c r="C64" t="s">
-        <v>10</v>
-      </c>
-      <c r="D64" t="s">
-        <v>11</v>
-      </c>
-      <c r="E64" t="s">
-        <v>17</v>
-      </c>
       <c r="F64" t="s">
-        <v>18</v>
+        <v>154</v>
       </c>
       <c r="G64" t="s">
-        <v>19</v>
+        <v>155</v>
       </c>
       <c r="H64" t="s">
         <v>34</v>
@@ -2651,7 +2693,7 @@
     </row>
     <row r="65">
       <c r="A65" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="B65" t="s">
         <v>9</v>
@@ -2660,50 +2702,50 @@
         <v>10</v>
       </c>
       <c r="D65" t="s">
-        <v>75</v>
+        <v>11</v>
       </c>
       <c r="E65" t="s">
-        <v>76</v>
+        <v>17</v>
       </c>
       <c r="F65" t="s">
-        <v>114</v>
+        <v>18</v>
       </c>
       <c r="G65" t="s">
-        <v>115</v>
+        <v>19</v>
       </c>
       <c r="H65" t="s">
-        <v>116</v>
+        <v>37</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="B66" t="s">
-        <v>9</v>
+        <v>34</v>
       </c>
       <c r="C66" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="D66" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="E66" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="F66" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="G66" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="H66" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="B67" t="s">
         <v>9</v>
@@ -2712,24 +2754,24 @@
         <v>10</v>
       </c>
       <c r="D67" t="s">
-        <v>84</v>
+        <v>11</v>
       </c>
       <c r="E67" t="s">
-        <v>85</v>
+        <v>17</v>
       </c>
       <c r="F67" t="s">
-        <v>157</v>
+        <v>18</v>
       </c>
       <c r="G67" t="s">
-        <v>28</v>
+        <v>19</v>
       </c>
       <c r="H67" t="s">
-        <v>28</v>
+        <v>20</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="B68" t="s">
         <v>9</v>
@@ -2738,97 +2780,97 @@
         <v>10</v>
       </c>
       <c r="D68" t="s">
-        <v>84</v>
+        <v>11</v>
       </c>
       <c r="E68" t="s">
-        <v>85</v>
+        <v>17</v>
       </c>
       <c r="F68" t="s">
-        <v>159</v>
+        <v>18</v>
       </c>
       <c r="G68" t="s">
-        <v>160</v>
+        <v>19</v>
       </c>
       <c r="H68" t="s">
-        <v>28</v>
+        <v>40</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B69" t="s">
-        <v>28</v>
+        <v>9</v>
       </c>
       <c r="C69" t="s">
-        <v>28</v>
+        <v>10</v>
       </c>
       <c r="D69" t="s">
         <v>28</v>
       </c>
       <c r="E69" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F69" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="G69" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="H69" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="B70" t="s">
         <v>9</v>
       </c>
       <c r="C70" t="s">
-        <v>10</v>
+        <v>34</v>
       </c>
       <c r="D70" t="s">
-        <v>75</v>
+        <v>34</v>
       </c>
       <c r="E70" t="s">
-        <v>76</v>
+        <v>34</v>
       </c>
       <c r="F70" t="s">
-        <v>114</v>
+        <v>34</v>
       </c>
       <c r="G70" t="s">
-        <v>115</v>
+        <v>34</v>
       </c>
       <c r="H70" t="s">
-        <v>116</v>
+        <v>34</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="s">
+        <v>162</v>
+      </c>
+      <c r="B71" t="s">
+        <v>9</v>
+      </c>
+      <c r="C71" t="s">
+        <v>10</v>
+      </c>
+      <c r="D71" t="s">
+        <v>96</v>
+      </c>
+      <c r="E71" t="s">
+        <v>97</v>
+      </c>
+      <c r="F71" t="s">
         <v>163</v>
       </c>
-      <c r="B71" t="s">
-        <v>9</v>
-      </c>
-      <c r="C71" t="s">
-        <v>10</v>
-      </c>
-      <c r="D71" t="s">
-        <v>11</v>
-      </c>
-      <c r="E71" t="s">
-        <v>17</v>
-      </c>
-      <c r="F71" t="s">
-        <v>18</v>
-      </c>
       <c r="G71" t="s">
-        <v>19</v>
+        <v>34</v>
       </c>
       <c r="H71" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
     </row>
     <row r="72">
@@ -2839,79 +2881,79 @@
         <v>9</v>
       </c>
       <c r="C72" t="s">
-        <v>37</v>
+        <v>10</v>
       </c>
       <c r="D72" t="s">
-        <v>38</v>
+        <v>96</v>
       </c>
       <c r="E72" t="s">
-        <v>106</v>
+        <v>97</v>
       </c>
       <c r="F72" t="s">
-        <v>107</v>
+        <v>165</v>
       </c>
       <c r="G72" t="s">
-        <v>108</v>
+        <v>166</v>
       </c>
       <c r="H72" t="s">
-        <v>165</v>
+        <v>34</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="B73" t="s">
         <v>9</v>
       </c>
       <c r="C73" t="s">
-        <v>10</v>
+        <v>168</v>
       </c>
       <c r="D73" t="s">
-        <v>22</v>
+        <v>169</v>
       </c>
       <c r="E73" t="s">
-        <v>51</v>
+        <v>170</v>
       </c>
       <c r="F73" t="s">
-        <v>52</v>
+        <v>171</v>
       </c>
       <c r="G73" t="s">
-        <v>53</v>
+        <v>172</v>
       </c>
       <c r="H73" t="s">
-        <v>28</v>
+        <v>173</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="s">
-        <v>167</v>
+        <v>174</v>
       </c>
       <c r="B74" t="s">
-        <v>9</v>
+        <v>34</v>
       </c>
       <c r="C74" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="D74" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="E74" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="F74" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="G74" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="H74" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="s">
-        <v>168</v>
+        <v>175</v>
       </c>
       <c r="B75" t="s">
         <v>9</v>
@@ -2920,24 +2962,24 @@
         <v>10</v>
       </c>
       <c r="D75" t="s">
-        <v>11</v>
+        <v>28</v>
       </c>
       <c r="E75" t="s">
-        <v>17</v>
+        <v>29</v>
       </c>
       <c r="F75" t="s">
-        <v>18</v>
+        <v>30</v>
       </c>
       <c r="G75" t="s">
-        <v>19</v>
+        <v>31</v>
       </c>
       <c r="H75" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="s">
-        <v>169</v>
+        <v>176</v>
       </c>
       <c r="B76" t="s">
         <v>9</v>
@@ -2946,102 +2988,102 @@
         <v>10</v>
       </c>
       <c r="D76" t="s">
-        <v>22</v>
+        <v>11</v>
       </c>
       <c r="E76" t="s">
-        <v>140</v>
+        <v>17</v>
       </c>
       <c r="F76" t="s">
-        <v>170</v>
+        <v>18</v>
       </c>
       <c r="G76" t="s">
-        <v>171</v>
+        <v>19</v>
       </c>
       <c r="H76" t="s">
-        <v>172</v>
+        <v>37</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="s">
-        <v>173</v>
+        <v>177</v>
       </c>
       <c r="B77" t="s">
         <v>9</v>
       </c>
       <c r="C77" t="s">
-        <v>10</v>
+        <v>45</v>
       </c>
       <c r="D77" t="s">
-        <v>11</v>
+        <v>46</v>
       </c>
       <c r="E77" t="s">
-        <v>17</v>
+        <v>118</v>
       </c>
       <c r="F77" t="s">
-        <v>18</v>
+        <v>119</v>
       </c>
       <c r="G77" t="s">
-        <v>19</v>
+        <v>120</v>
       </c>
       <c r="H77" t="s">
-        <v>28</v>
+        <v>178</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
       <c r="B78" t="s">
         <v>9</v>
       </c>
       <c r="C78" t="s">
-        <v>28</v>
+        <v>10</v>
       </c>
       <c r="D78" t="s">
-        <v>28</v>
+        <v>22</v>
       </c>
       <c r="E78" t="s">
-        <v>28</v>
+        <v>59</v>
       </c>
       <c r="F78" t="s">
-        <v>28</v>
+        <v>60</v>
       </c>
       <c r="G78" t="s">
-        <v>28</v>
+        <v>61</v>
       </c>
       <c r="H78" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="B79" t="s">
         <v>9</v>
       </c>
       <c r="C79" t="s">
-        <v>10</v>
+        <v>34</v>
       </c>
       <c r="D79" t="s">
-        <v>11</v>
+        <v>34</v>
       </c>
       <c r="E79" t="s">
-        <v>17</v>
+        <v>34</v>
       </c>
       <c r="F79" t="s">
-        <v>18</v>
+        <v>34</v>
       </c>
       <c r="G79" t="s">
-        <v>19</v>
+        <v>34</v>
       </c>
       <c r="H79" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="B80" t="s">
         <v>9</v>
@@ -3062,12 +3104,12 @@
         <v>19</v>
       </c>
       <c r="H80" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="s">
-        <v>177</v>
+        <v>182</v>
       </c>
       <c r="B81" t="s">
         <v>9</v>
@@ -3076,24 +3118,24 @@
         <v>10</v>
       </c>
       <c r="D81" t="s">
-        <v>11</v>
+        <v>22</v>
       </c>
       <c r="E81" t="s">
-        <v>17</v>
+        <v>146</v>
       </c>
       <c r="F81" t="s">
-        <v>18</v>
+        <v>183</v>
       </c>
       <c r="G81" t="s">
-        <v>19</v>
+        <v>184</v>
       </c>
       <c r="H81" t="s">
-        <v>178</v>
+        <v>185</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="s">
-        <v>179</v>
+        <v>186</v>
       </c>
       <c r="B82" t="s">
         <v>9</v>
@@ -3114,64 +3156,64 @@
         <v>19</v>
       </c>
       <c r="H82" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="s">
-        <v>180</v>
+        <v>187</v>
       </c>
       <c r="B83" t="s">
-        <v>28</v>
+        <v>9</v>
       </c>
       <c r="C83" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="D83" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="E83" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="F83" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="G83" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="H83" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="s">
-        <v>181</v>
+        <v>188</v>
       </c>
       <c r="B84" t="s">
-        <v>28</v>
+        <v>9</v>
       </c>
       <c r="C84" t="s">
-        <v>28</v>
+        <v>10</v>
       </c>
       <c r="D84" t="s">
-        <v>28</v>
+        <v>11</v>
       </c>
       <c r="E84" t="s">
-        <v>28</v>
+        <v>17</v>
       </c>
       <c r="F84" t="s">
-        <v>28</v>
+        <v>18</v>
       </c>
       <c r="G84" t="s">
-        <v>28</v>
+        <v>19</v>
       </c>
       <c r="H84" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="s">
-        <v>182</v>
+        <v>189</v>
       </c>
       <c r="B85" t="s">
         <v>9</v>
@@ -3192,12 +3234,12 @@
         <v>19</v>
       </c>
       <c r="H85" t="s">
-        <v>178</v>
+        <v>37</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="s">
-        <v>183</v>
+        <v>190</v>
       </c>
       <c r="B86" t="s">
         <v>9</v>
@@ -3218,12 +3260,12 @@
         <v>19</v>
       </c>
       <c r="H86" t="s">
-        <v>31</v>
+        <v>191</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="s">
-        <v>184</v>
+        <v>192</v>
       </c>
       <c r="B87" t="s">
         <v>9</v>
@@ -3232,76 +3274,76 @@
         <v>10</v>
       </c>
       <c r="D87" t="s">
-        <v>84</v>
+        <v>11</v>
       </c>
       <c r="E87" t="s">
-        <v>85</v>
+        <v>17</v>
       </c>
       <c r="F87" t="s">
-        <v>157</v>
+        <v>18</v>
       </c>
       <c r="G87" t="s">
-        <v>28</v>
+        <v>19</v>
       </c>
       <c r="H87" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="s">
-        <v>185</v>
+        <v>193</v>
       </c>
       <c r="B88" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="C88" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="D88" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="E88" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="F88" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="G88" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="H88" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="s">
-        <v>186</v>
+        <v>194</v>
       </c>
       <c r="B89" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="C89" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="D89" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="E89" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="F89" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="G89" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="H89" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="s">
-        <v>187</v>
+        <v>195</v>
       </c>
       <c r="B90" t="s">
         <v>9</v>
@@ -3322,38 +3364,38 @@
         <v>19</v>
       </c>
       <c r="H90" t="s">
-        <v>31</v>
+        <v>191</v>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="s">
-        <v>188</v>
+        <v>196</v>
       </c>
       <c r="B91" t="s">
         <v>9</v>
       </c>
       <c r="C91" t="s">
-        <v>28</v>
+        <v>10</v>
       </c>
       <c r="D91" t="s">
-        <v>28</v>
+        <v>11</v>
       </c>
       <c r="E91" t="s">
-        <v>28</v>
+        <v>17</v>
       </c>
       <c r="F91" t="s">
-        <v>28</v>
+        <v>18</v>
       </c>
       <c r="G91" t="s">
-        <v>28</v>
+        <v>19</v>
       </c>
       <c r="H91" t="s">
-        <v>28</v>
+        <v>37</v>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="s">
-        <v>189</v>
+        <v>197</v>
       </c>
       <c r="B92" t="s">
         <v>9</v>
@@ -3362,128 +3404,128 @@
         <v>10</v>
       </c>
       <c r="D92" t="s">
-        <v>11</v>
+        <v>96</v>
       </c>
       <c r="E92" t="s">
-        <v>17</v>
+        <v>97</v>
       </c>
       <c r="F92" t="s">
-        <v>18</v>
+        <v>163</v>
       </c>
       <c r="G92" t="s">
-        <v>19</v>
+        <v>34</v>
       </c>
       <c r="H92" t="s">
-        <v>190</v>
+        <v>34</v>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="s">
-        <v>191</v>
+        <v>198</v>
       </c>
       <c r="B93" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="C93" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="D93" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="E93" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="F93" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="G93" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="H93" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="s">
-        <v>192</v>
+        <v>199</v>
       </c>
       <c r="B94" t="s">
-        <v>9</v>
+        <v>34</v>
       </c>
       <c r="C94" t="s">
-        <v>10</v>
+        <v>34</v>
       </c>
       <c r="D94" t="s">
-        <v>75</v>
+        <v>34</v>
       </c>
       <c r="E94" t="s">
-        <v>76</v>
+        <v>34</v>
       </c>
       <c r="F94" t="s">
-        <v>77</v>
+        <v>34</v>
       </c>
       <c r="G94" t="s">
-        <v>78</v>
+        <v>34</v>
       </c>
       <c r="H94" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="s">
-        <v>193</v>
+        <v>200</v>
       </c>
       <c r="B95" t="s">
-        <v>28</v>
+        <v>9</v>
       </c>
       <c r="C95" t="s">
-        <v>28</v>
+        <v>10</v>
       </c>
       <c r="D95" t="s">
-        <v>28</v>
+        <v>11</v>
       </c>
       <c r="E95" t="s">
-        <v>28</v>
+        <v>17</v>
       </c>
       <c r="F95" t="s">
-        <v>28</v>
+        <v>18</v>
       </c>
       <c r="G95" t="s">
-        <v>28</v>
+        <v>19</v>
       </c>
       <c r="H95" t="s">
-        <v>28</v>
+        <v>37</v>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="s">
-        <v>194</v>
+        <v>201</v>
       </c>
       <c r="B96" t="s">
         <v>9</v>
       </c>
       <c r="C96" t="s">
-        <v>10</v>
+        <v>34</v>
       </c>
       <c r="D96" t="s">
-        <v>11</v>
+        <v>34</v>
       </c>
       <c r="E96" t="s">
-        <v>17</v>
+        <v>34</v>
       </c>
       <c r="F96" t="s">
-        <v>18</v>
+        <v>34</v>
       </c>
       <c r="G96" t="s">
-        <v>19</v>
+        <v>34</v>
       </c>
       <c r="H96" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="s">
-        <v>195</v>
+        <v>202</v>
       </c>
       <c r="B97" t="s">
         <v>9</v>
@@ -3504,38 +3546,38 @@
         <v>19</v>
       </c>
       <c r="H97" t="s">
-        <v>34</v>
+        <v>203</v>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="s">
-        <v>196</v>
+        <v>204</v>
       </c>
       <c r="B98" t="s">
-        <v>9</v>
+        <v>34</v>
       </c>
       <c r="C98" t="s">
-        <v>10</v>
+        <v>34</v>
       </c>
       <c r="D98" t="s">
-        <v>11</v>
+        <v>34</v>
       </c>
       <c r="E98" t="s">
-        <v>17</v>
+        <v>34</v>
       </c>
       <c r="F98" t="s">
-        <v>18</v>
+        <v>34</v>
       </c>
       <c r="G98" t="s">
-        <v>19</v>
+        <v>34</v>
       </c>
       <c r="H98" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="s">
-        <v>197</v>
+        <v>205</v>
       </c>
       <c r="B99" t="s">
         <v>9</v>
@@ -3544,42 +3586,42 @@
         <v>10</v>
       </c>
       <c r="D99" t="s">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="E99" t="s">
-        <v>23</v>
+        <v>29</v>
       </c>
       <c r="F99" t="s">
-        <v>198</v>
+        <v>83</v>
       </c>
       <c r="G99" t="s">
-        <v>199</v>
+        <v>84</v>
       </c>
       <c r="H99" t="s">
-        <v>200</v>
+        <v>34</v>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="s">
-        <v>201</v>
+        <v>206</v>
       </c>
       <c r="B100" t="s">
-        <v>9</v>
+        <v>34</v>
       </c>
       <c r="C100" t="s">
-        <v>10</v>
+        <v>34</v>
       </c>
       <c r="D100" t="s">
-        <v>11</v>
+        <v>34</v>
       </c>
       <c r="E100" t="s">
-        <v>17</v>
+        <v>34</v>
       </c>
       <c r="F100" t="s">
-        <v>18</v>
+        <v>34</v>
       </c>
       <c r="G100" t="s">
-        <v>19</v>
+        <v>34</v>
       </c>
       <c r="H100" t="s">
         <v>34</v>
@@ -3587,7 +3629,7 @@
     </row>
     <row r="101">
       <c r="A101" t="s">
-        <v>202</v>
+        <v>207</v>
       </c>
       <c r="B101" t="s">
         <v>9</v>
@@ -3608,38 +3650,38 @@
         <v>19</v>
       </c>
       <c r="H101" t="s">
-        <v>178</v>
+        <v>37</v>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="s">
-        <v>203</v>
+        <v>208</v>
       </c>
       <c r="B102" t="s">
-        <v>28</v>
+        <v>9</v>
       </c>
       <c r="C102" t="s">
-        <v>28</v>
+        <v>10</v>
       </c>
       <c r="D102" t="s">
-        <v>28</v>
+        <v>11</v>
       </c>
       <c r="E102" t="s">
-        <v>28</v>
+        <v>17</v>
       </c>
       <c r="F102" t="s">
-        <v>28</v>
+        <v>18</v>
       </c>
       <c r="G102" t="s">
-        <v>28</v>
+        <v>19</v>
       </c>
       <c r="H102" t="s">
-        <v>28</v>
+        <v>40</v>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="s">
-        <v>204</v>
+        <v>209</v>
       </c>
       <c r="B103" t="s">
         <v>9</v>
@@ -3648,50 +3690,50 @@
         <v>10</v>
       </c>
       <c r="D103" t="s">
-        <v>75</v>
+        <v>11</v>
       </c>
       <c r="E103" t="s">
-        <v>76</v>
+        <v>17</v>
       </c>
       <c r="F103" t="s">
-        <v>28</v>
+        <v>18</v>
       </c>
       <c r="G103" t="s">
-        <v>28</v>
+        <v>19</v>
       </c>
       <c r="H103" t="s">
-        <v>28</v>
+        <v>37</v>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="s">
-        <v>205</v>
+        <v>210</v>
       </c>
       <c r="B104" t="s">
-        <v>28</v>
+        <v>9</v>
       </c>
       <c r="C104" t="s">
-        <v>28</v>
+        <v>10</v>
       </c>
       <c r="D104" t="s">
-        <v>28</v>
+        <v>22</v>
       </c>
       <c r="E104" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="F104" t="s">
-        <v>28</v>
+        <v>211</v>
       </c>
       <c r="G104" t="s">
-        <v>28</v>
+        <v>212</v>
       </c>
       <c r="H104" t="s">
-        <v>28</v>
+        <v>213</v>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="s">
-        <v>206</v>
+        <v>214</v>
       </c>
       <c r="B105" t="s">
         <v>9</v>
@@ -3712,134 +3754,134 @@
         <v>19</v>
       </c>
       <c r="H105" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="s">
-        <v>207</v>
+        <v>215</v>
       </c>
       <c r="B106" t="s">
-        <v>9</v>
+        <v>34</v>
       </c>
       <c r="C106" t="s">
-        <v>10</v>
+        <v>34</v>
       </c>
       <c r="D106" t="s">
-        <v>75</v>
+        <v>34</v>
       </c>
       <c r="E106" t="s">
-        <v>76</v>
+        <v>34</v>
       </c>
       <c r="F106" t="s">
-        <v>208</v>
+        <v>34</v>
       </c>
       <c r="G106" t="s">
-        <v>209</v>
+        <v>34</v>
       </c>
       <c r="H106" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="s">
-        <v>210</v>
+        <v>216</v>
       </c>
       <c r="B107" t="s">
         <v>9</v>
       </c>
       <c r="C107" t="s">
-        <v>28</v>
+        <v>10</v>
       </c>
       <c r="D107" t="s">
-        <v>28</v>
+        <v>11</v>
       </c>
       <c r="E107" t="s">
-        <v>28</v>
+        <v>17</v>
       </c>
       <c r="F107" t="s">
-        <v>28</v>
+        <v>18</v>
       </c>
       <c r="G107" t="s">
-        <v>28</v>
+        <v>19</v>
       </c>
       <c r="H107" t="s">
-        <v>28</v>
+        <v>191</v>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="s">
-        <v>211</v>
+        <v>217</v>
       </c>
       <c r="B108" t="s">
-        <v>9</v>
+        <v>34</v>
       </c>
       <c r="C108" t="s">
-        <v>10</v>
+        <v>34</v>
       </c>
       <c r="D108" t="s">
-        <v>11</v>
+        <v>34</v>
       </c>
       <c r="E108" t="s">
-        <v>17</v>
+        <v>34</v>
       </c>
       <c r="F108" t="s">
-        <v>18</v>
+        <v>34</v>
       </c>
       <c r="G108" t="s">
-        <v>19</v>
+        <v>34</v>
       </c>
       <c r="H108" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="s">
-        <v>212</v>
+        <v>218</v>
       </c>
       <c r="B109" t="s">
-        <v>28</v>
+        <v>9</v>
       </c>
       <c r="C109" t="s">
-        <v>28</v>
+        <v>10</v>
       </c>
       <c r="D109" t="s">
         <v>28</v>
       </c>
       <c r="E109" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F109" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="G109" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="H109" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="s">
-        <v>213</v>
+        <v>219</v>
       </c>
       <c r="B110" t="s">
-        <v>9</v>
+        <v>34</v>
       </c>
       <c r="C110" t="s">
-        <v>10</v>
+        <v>34</v>
       </c>
       <c r="D110" t="s">
-        <v>11</v>
+        <v>34</v>
       </c>
       <c r="E110" t="s">
-        <v>17</v>
+        <v>34</v>
       </c>
       <c r="F110" t="s">
-        <v>18</v>
+        <v>34</v>
       </c>
       <c r="G110" t="s">
-        <v>19</v>
+        <v>34</v>
       </c>
       <c r="H110" t="s">
         <v>34</v>
@@ -3847,7 +3889,7 @@
     </row>
     <row r="111">
       <c r="A111" t="s">
-        <v>214</v>
+        <v>220</v>
       </c>
       <c r="B111" t="s">
         <v>9</v>
@@ -3856,19 +3898,175 @@
         <v>10</v>
       </c>
       <c r="D111" t="s">
+        <v>11</v>
+      </c>
+      <c r="E111" t="s">
+        <v>17</v>
+      </c>
+      <c r="F111" t="s">
+        <v>18</v>
+      </c>
+      <c r="G111" t="s">
+        <v>19</v>
+      </c>
+      <c r="H111" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="s">
+        <v>221</v>
+      </c>
+      <c r="B112" t="s">
+        <v>9</v>
+      </c>
+      <c r="C112" t="s">
+        <v>10</v>
+      </c>
+      <c r="D112" t="s">
+        <v>28</v>
+      </c>
+      <c r="E112" t="s">
+        <v>29</v>
+      </c>
+      <c r="F112" t="s">
+        <v>222</v>
+      </c>
+      <c r="G112" t="s">
+        <v>223</v>
+      </c>
+      <c r="H112" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="s">
+        <v>224</v>
+      </c>
+      <c r="B113" t="s">
+        <v>9</v>
+      </c>
+      <c r="C113" t="s">
+        <v>34</v>
+      </c>
+      <c r="D113" t="s">
+        <v>34</v>
+      </c>
+      <c r="E113" t="s">
+        <v>34</v>
+      </c>
+      <c r="F113" t="s">
+        <v>34</v>
+      </c>
+      <c r="G113" t="s">
+        <v>34</v>
+      </c>
+      <c r="H113" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="s">
+        <v>225</v>
+      </c>
+      <c r="B114" t="s">
+        <v>9</v>
+      </c>
+      <c r="C114" t="s">
+        <v>10</v>
+      </c>
+      <c r="D114" t="s">
+        <v>11</v>
+      </c>
+      <c r="E114" t="s">
+        <v>17</v>
+      </c>
+      <c r="F114" t="s">
+        <v>18</v>
+      </c>
+      <c r="G114" t="s">
+        <v>19</v>
+      </c>
+      <c r="H114" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="s">
+        <v>226</v>
+      </c>
+      <c r="B115" t="s">
+        <v>34</v>
+      </c>
+      <c r="C115" t="s">
+        <v>34</v>
+      </c>
+      <c r="D115" t="s">
+        <v>34</v>
+      </c>
+      <c r="E115" t="s">
+        <v>34</v>
+      </c>
+      <c r="F115" t="s">
+        <v>34</v>
+      </c>
+      <c r="G115" t="s">
+        <v>34</v>
+      </c>
+      <c r="H115" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="s">
+        <v>227</v>
+      </c>
+      <c r="B116" t="s">
+        <v>9</v>
+      </c>
+      <c r="C116" t="s">
+        <v>10</v>
+      </c>
+      <c r="D116" t="s">
+        <v>11</v>
+      </c>
+      <c r="E116" t="s">
+        <v>17</v>
+      </c>
+      <c r="F116" t="s">
+        <v>18</v>
+      </c>
+      <c r="G116" t="s">
+        <v>19</v>
+      </c>
+      <c r="H116" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="s">
+        <v>228</v>
+      </c>
+      <c r="B117" t="s">
+        <v>9</v>
+      </c>
+      <c r="C117" t="s">
+        <v>10</v>
+      </c>
+      <c r="D117" t="s">
         <v>22</v>
       </c>
-      <c r="E111" t="s">
-        <v>51</v>
-      </c>
-      <c r="F111" t="s">
-        <v>52</v>
-      </c>
-      <c r="G111" t="s">
-        <v>53</v>
-      </c>
-      <c r="H111" t="s">
-        <v>118</v>
+      <c r="E117" t="s">
+        <v>59</v>
+      </c>
+      <c r="F117" t="s">
+        <v>60</v>
+      </c>
+      <c r="G117" t="s">
+        <v>61</v>
+      </c>
+      <c r="H117" t="s">
+        <v>127</v>
       </c>
     </row>
   </sheetData>

</xml_diff>